<commit_message>
updated excel sheet generator, error fixed
</commit_message>
<xml_diff>
--- a/static/auto_sheets/Field Samples Meta Data Requirements and Template.xlsx
+++ b/static/auto_sheets/Field Samples Meta Data Requirements and Template.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,7 +500,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Broad-Scale Environmental Context</t>
+          <t>Local Environmental Context</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -513,16 +513,32 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>litter layer</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>canopy</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Report the entity or entities which are in the sample or specimen’s local vicinity and which you believe have significant causal influences on your sample or specimen. We recommend using EnvO terms which are of smaller spatial grain than your entry for env_broad_scale. Terms, such as anatomical sites, from other OBO Library ontologies which interoperate with EnvO (e.g. UBERON) are accepted in this field. EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS. Multiple values allowed if seperated by semi-colon.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sample storage location</t>
+          <t>Environmental Medium</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -537,34 +553,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>A: shelf 4.5; W: shelf 4.6</t>
+          <t>Soil</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A: shelf 4.5; W: shelf 4.6</t>
+          <t>Ocean water</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>A: shelf 4.5; W: shelf 4.6</t>
+          <t>pond water</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">If working half and archive half are stored different places, report two locations seperated by semi-colon and preceded by either A: or W: </t>
+          <t>Report the environmental material(s) immediately surrounding the sample or specimen at the time of sampling. We recommend using subclasses of "environmental material" (http://purl.obolibrary.org/obo/ENVO_00010483). EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS . Terms from other OBO ontologies are permissible as long as they reference mass/volume nouns (e.g. air, water, blood) and not discrete, countable entities (e.g. a tree, a leaf, a table top).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sample storage setting</t>
+          <t>Broad-Scale Environmental Context</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -577,36 +593,20 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Cold room</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Walk-in Freezer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Cold room</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Specify the storage setting </t>
+          <t>Report the major environmental system the sample or specimen came from. The system(s) identified should have a coarse spatial grain, to provide the general environmental context of where the sampling was done (e.g. in the desert or a rainforest). We recommend using subclasses of EnvO’s biome class:  http://purl.obolibrary.org/obo/ENVO_00000428. EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sample storage address</t>
+          <t>Sample storage location</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -621,39 +621,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>A: shelf 4.5; W: shelf 4.6</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Address </t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>The exact address where the sample. If it's stored at geological museum then you can just write "GM".</t>
+          <t xml:space="preserve">If working half and archive half are stored different places, report two locations seperated by semi-colon and preceded by either A: or W: </t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Elevation (meters)</t>
+          <t>Sample storage setting</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -661,32 +661,36 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>37</v>
-      </c>
-      <c r="E7" t="n">
-        <v>37</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Cold room</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Walk-in Freezer</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>37.5</t>
+          <t>Cold room</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Number (decimal allowed)</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Vertical height above mean sea level. Specify as negative number if below mean sea level.</t>
+          <t xml:space="preserve">Specify the storage setting </t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Environmental Medium</t>
+          <t>Sample storage address</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -699,21 +703,41 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Address </t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>The exact address where the sample is stored. If it's stored at geological museum then you can just write "GM".</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sample type</t>
+          <t>Elevation (meters)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -721,41 +745,37 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Fossil</t>
-        </is>
+      <c r="D9" t="n">
+        <v>37</v>
+      </c>
+      <c r="E9" t="n">
+        <v>37</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>OSL</t>
+          <t>37.5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mathematical notation: Numbers, "()", "[]" and "," (decimal allowed only if "." is used as decimal point).</t>
+          <t>Number (decimal allowed)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Container used for sample collection/extraction/excavation</t>
+          <t>Vertical height above mean sea level. Specify as negative number if below mean sea level.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Water depth (m)</t>
+          <t>Site Type</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -763,24 +783,36 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Outcrop</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Cave</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Lake</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Decimal numbers or integers</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Depth below surface of water body, from where the sample was taken</t>
+          <t>The type of site the sediment cores where taken. E.g. ocean, marine, freshwater, brackish, ice caves, caves. We recommend using terms from the EnvO ontology: http://environmentontology.org/ to ensure data consistency.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Site Type</t>
+          <t>Sample type</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -795,39 +827,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Outcrop</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cave</t>
+          <t>Fossil</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Lake</t>
+          <t>OSL</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>The type of site the sediment cores where taken. E.g. ocean, marine, freshwater, brackish, ice caves, caves. Please use ENVO ontology: http://environmentontology.org/</t>
+          <t>Report the type of sample. Please choose among a predefined set of sample types, to ensure consistency.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Local Environmental Context</t>
+          <t>Water depth (m)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -838,18 +870,26 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Decimal numbers or integers</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Depth below surface of water body, from where the sample was taken</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Longitude</t>
+          <t>Sample Supertype</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -857,35 +897,37 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>-45.5347</v>
-      </c>
-      <c r="E13" t="n">
-        <v>-45.5347</v>
-      </c>
-      <c r="F13" t="n">
-        <v>-45.5347</v>
-      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>discrete</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>continous</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>decimal degrees, max 3 digits, max 8 decimal points (-180 to 180)</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>The geographical origin of the sample as defined by longitude. The values should be reported in decimal degrees as precise as possible (max. 8 decimal points).</t>
+          <t>Report wether the sample is discrete or continous. A discrete field sample is defined as a sample where any sub-samples derived from it retain identical metadata to the original parent sample, except for volume and/or weight. For instance, if you take a subsample of an Archive Sample, it will (should) maintain the same depth and age as the parent sample. A continous sample however is a sample that can have multiple unique subsamples in terms of one or more parameters.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Country/Ocean</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -893,35 +935,41 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>61.1399</v>
-      </c>
-      <c r="E14" t="n">
-        <v>61.1399</v>
-      </c>
-      <c r="F14" t="n">
-        <v>61.1399</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Greenland</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>decimal degrees using WGS84 GPS Standard. Max 2 digits, max 8 decimal points (-90 to 90)</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>The geographical origin of the sample as defined by latitude.</t>
+          <t>The geographical origin of the sample as defined by the country or sea name. Country or sea names should be chosen from the INSDC country list (http://insdc.org/country.html), or the GAZ ontology (http://purl.bioontology.org/ontology/GAZ)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Country/Ocean</t>
+          <t>Longitude</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -929,67 +977,71 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Greenland</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
+      <c r="D15" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-45.5347</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-45.5347</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>decimal degrees in WGS84 system, max 3 digits, max 8 decimal points (-180 to 180)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>The geographical origin of the sample as defined by the country or sea name. Country or sea names should be chosen from the INSDC country list (http://insdc.org/country.html), or the GAZ ontology (http://purl.bioontology.org/ontology/GAZ)</t>
+          <t>The geographical origin of the sample as defined by longitude. The values should be reported in decimal degrees and in WGS84 system as precise as possible (max. 8 decimal points).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>QR Code</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="E16" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="F16" t="n">
+        <v>61.1399</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>decimal degrees using WGS84 GPS Standard. Max 2 digits, max 8 decimal points (-90 to 90)</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>An id for the physical QR code on the sample</t>
+          <t>The geographical origin of the sample as defined by latitude using decimal degrees and in WGS84 system.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Region/Province/State</t>
+          <t>Sampling depth (discrete, cm)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>double precision</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -997,21 +1049,37 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" t="n">
+        <v>200</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>300.3</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Numbers (decimals allowed)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Depth measurement for discrete type samples (such as tube). Only fill this out if your sample type is discrete. If the sample is continous, use columns "Sampling depth (top, cm)" and "Sampling depth (bottom, cm)". Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Age Estimate (to, KABP)</t>
+          <t>QR Code</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1019,37 +1087,25 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>litter layer</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>canopy</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Report the entity or entities which are in the sample or specimen’s local vicinity and which you believe have significant causal influences on your sample or specimen. We recommend using EnvO terms which are of smaller spatial grain than your entry for env_broad_scale. Terms, such as anatomical sites, from other OBO Library ontologies which interoperate with EnvO (e.g. UBERON) are accepted in this field. EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS. Multiple values allowed if seperated by semi-colon.</t>
+          <t>An id for the physical QR code on the sample</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sampling depth estimation (bottom, cm)</t>
+          <t>City/Town/Lake/Location</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1059,17 +1115,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Soul</t>
+          <t>Hollerup</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ocean water</t>
+          <t>Hollerup</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>pond water</t>
+          <t>Hollerup</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1079,14 +1135,14 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Report the environmental material(s) immediately surrounding the sample or specimen at the time of sampling. We recommend using subclasses of "environmental material" (http://purl.obolibrary.org/obo/ENVO_00010483). EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS . Terms from other OBO ontologies are permissible as long as they reference mass/volume nouns (e.g. air, water, blood) and not discrete, countable entities (e.g. a tree, a leaf, a table top).</t>
+          <t>If relevant. Otherwise leave blank.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Comment</t>
+          <t>Region/Province/State</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1099,25 +1155,41 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Hollerup</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> The geographical origin of the sample as defined by the region/province/state. If relevant. Otherwise leave blank.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Link to other relevant data</t>
+          <t>Age Estimate (to, KABP)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1125,29 +1197,41 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>105</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1105</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Link to other relevant data.</t>
+          <t>Not precise, just an estimate. Remember to fill out the "from" value as well. ACCEPTED UNIT: Kilo annum before present (1950).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Link to images</t>
+          <t>Sampling depth estimation (bottom, cm)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1155,24 +1239,36 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-10</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>Integers and minus sign</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Link to any relevant images of the sample.</t>
+          <t>Depth measurement as measured from the bottom of the sample. Only for interval type samples (such as core). DO NOT FILL if your sample is discrete. Use column "Sampling depth (discrete, cm)" instead. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Miscellaneous Environmental Measurements or Observations</t>
+          <t>Comment</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1185,36 +1281,20 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">temperature: 7 celcius; </t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">temperature: 7 celcius; </t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>temperature: 7 celcius; cloud cover: overcast;</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Any other relevant environmental measurements/observations. If multiple: seperate by semi-colon.</t>
-        </is>
-      </c>
+          <t>text and/or numbers</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Miscellaneous Sample Measurements or Observations</t>
+          <t>Link to other relevant data</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1227,41 +1307,29 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">water content: 10 %; </t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>water content: 10 %;</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>water content: 10 %; porosity: 5 %</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Any relevant measurements/observations taken of the field sample. If multiple: seperate by semi-colon.</t>
+          <t>Link to other relevant data.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Disposal date</t>
+          <t>Link to images</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1269,41 +1337,29 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2023-10-22</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2023-10-22</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>2023-10-22</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Report when the sample was disposed.</t>
+          <t>Link to any relevant images of the sample.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Storing date</t>
+          <t>Miscellaneous Environmental Measurements or Observations</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1313,34 +1369,34 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t xml:space="preserve">temperature: 7 celcius; </t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t xml:space="preserve">temperature: 7 celcius; </t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>temperature: 7 celcius; cloud cover: overcast;</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Report when the sample was stored in the specified storage location.</t>
+          <t>Any other relevant environmental measurements/observations. If multiple: seperate by semi-colon.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Miscellaneous Sample Measurements or Observations</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1355,39 +1411,39 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t xml:space="preserve">water content: 10 %; </t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>water content: 10 %;</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>NOVO</t>
+          <t>water content: 10 %; porosity: 5 %</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>&lt;measurement/observation type&gt;: &lt;measurement/observation&gt; &lt;unit (optional)&gt;</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Specify the grant that funds the project.</t>
+          <t>Any relevant measurements/observations taken of the field sample. If multiple: seperate by semi-colon.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PI (KU ID)</t>
+          <t>Disposal date</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1397,39 +1453,39 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KU Id</t>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>KU id of the principal investigator responsible for the project.</t>
+          <t>Report when the sample was disposed.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Age Estimate (from, KABP)</t>
+          <t>Sampling Site</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1437,36 +1493,24 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>1105</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Not precise, just an estimate. Remember to fill out the "from" value as well. ACCEPTED UNIT: Kilo annum before present (1950).</t>
+          <t>Any other geographic location identifier that might be relevant. If the sample was taken from a known archeological site for example. Otherwise leave blank.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Period Estimate</t>
+          <t>Running Project Title</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1481,35 +1525,39 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Holocene</t>
+          <t>Traversing European Coastlines</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Holocene</t>
+          <t>Arctic Canada</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Pleistocene</t>
+          <t>Arctic Canada</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Full names seperated by comma</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>text and/or numbers</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Referencing this google sheet: https://docs.google.com/spreadsheets/d/10TWDtKMug4yzOQUP7Q4APIoPNHQXCFX_RasijIgyCAA/edit?usp=sharing</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Marine isotope stage estimate</t>
+          <t>Sampling Date</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1519,35 +1567,39 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>5e</t>
+          <t>2023-10-22</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Date when the sampling occured.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Sediment type</t>
+          <t>Age Estimate (from, KABP)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1557,39 +1609,39 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Lacustrine</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Glaciofluvial</t>
+          <t>105</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Glaciofluvial</t>
+          <t>1105</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Eg. Glacial, Lacustrine, Fluvial, Aeolian, Peat, Soil</t>
+          <t>Not precise, just an estimate. Remember to fill out the "to" value as well. ACCEPTED UNIT: Kilo annum before present (1950).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Sampling Date</t>
+          <t>Period Estimate</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1599,39 +1651,35 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>Holocene</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>Holocene</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2023-10-22</t>
+          <t>Pleistocene</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Date when the sampling occured.</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Correlation depth (top, cm)</t>
+          <t>Sampling Method</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1639,37 +1687,37 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>10</v>
-      </c>
-      <c r="E34" t="n">
-        <v>200</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>300.3</t>
-        </is>
-      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Coring</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Drilling</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Numbers (decimals allowed)</t>
+          <t>text</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>The local core depth  that correlates with the  correlation depth (bottom) of the core immediately below.</t>
+          <t>Report the sampling method used.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Correlation depth (bottom, cm)</t>
+          <t>Sample provider(s)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>numeric</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1677,32 +1725,36 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>10</v>
-      </c>
-      <c r="E35" t="n">
-        <v>200</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>hlj234</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>300.3</t>
+          <t>hlj234; glj523</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Numbers (decimals allowed)</t>
+          <t>KU Ids seperated by semicolon if multiple.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>The local core depth that correlates with the  correlation depth (top) of the core immediately above.</t>
+          <t>Unique KU id(s) of the person(s) responsible for the sample extraction, seperated by semicolon if multiple.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Sample provider(s)</t>
+          <t>Sediment type</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1717,39 +1769,39 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>Lacustrine</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>hlj234</t>
+          <t>Glaciofluvial</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>hlj234; glj523</t>
+          <t>Glaciofluvial</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KU Ids</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Unique KU id(s) of the person(s) responsible for the sample extraction, seperated by semicolon if multiple.</t>
+          <t>Eg. Glacial, Lacustrine, Fluvial, Aeolian, Peat, Soil</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sampling depth estimation (top, cm)</t>
+          <t>PI (KU ID)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1759,39 +1811,39 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>hlj234</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>hlj234</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>-10</t>
+          <t>hlj234</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Integers and minus sign</t>
+          <t>KU Id</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Depth measurement as measured from the top of the sample. Only for interval type samples (such as core). DO NOT FILL if your sample is discrete. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+          <t>KU id of the principal investigator responsible for the project.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sampling depth (discrete, cm)</t>
+          <t>Correlation depth (top, cm)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>double precision</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1817,19 +1869,19 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Depth measurement for discrete type samples (such as tube). Only fill this out if your sample type is discrete. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+          <t>The local core depth  that correlates with the  correlation depth (bottom) of the core immediately below.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Running Project Title</t>
+          <t>Correlation depth (bottom, cm)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>numeric</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1837,36 +1889,32 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Traversing European Coastlines</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Arctic Canada</t>
-        </is>
+      <c r="D39" t="n">
+        <v>10</v>
+      </c>
+      <c r="E39" t="n">
+        <v>200</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Arctic Canada</t>
+          <t>300.3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>text and/or numbers</t>
+          <t>Numbers (decimals allowed)</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Referencing this google sheet: https://docs.google.com/spreadsheets/d/10TWDtKMug4yzOQUP7Q4APIoPNHQXCFX_RasijIgyCAA/edit?usp=sharing</t>
+          <t>The local core depth that correlates with the  correlation depth (top) of the core immediately above.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>City/Town/Lake/Location</t>
+          <t>Grant</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1881,39 +1929,39 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Hollerup</t>
+          <t>NOVO</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>text and/or numbers</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>If relevant. Otherwise leave blank.</t>
+          <t>Specify the grant that funds the project.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Sampling Site</t>
+          <t>Sampling depth estimation (top, cm)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1921,123 +1969,111 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>-10</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
+          <t>Integers and minus sign</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Depth measurement as measured from the top of the sample. Only for interval type samples (such as core). DO NOT FILL if your sample is discrete. In that case fill column "Sampling depth (discrete, cm)". Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Storing date</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2023-10-22</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD or DD-MM-YYYY (choose one)</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Report when the sample was stored in the specified storage location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Marine isotope stage estimate</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>5e</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>text and/or numbers</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Any other geographic location identifier that might be relevant. If the sample was taken from a known archeological site for example. Otherwise leave blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>-10</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Integers and minus sign</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Depth measurement as measured from the bottom of the sample. Only for interval type samples (such as core). DO NOT FILL if your sample is discrete. Depth is defined as the vertical distance below local surface, e.g. for sediment or soil samples depth is measured from sediment or soil surface, respectively.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>1105</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Integer</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Not precise, just an estimate. Remember to fill out the "from" value as well. ACCEPTED UNIT: Kilo annum before present (1950).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Hollerup</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Hollerup</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Hollerup</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> The geographical origin of the sample as defined by the region/province/state. If relevant. Otherwise leave blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Report the major environmental system the sample or specimen came from. The system(s) identified should have a coarse spatial grain, to provide the general environmental context of where the sampling was done (e.g. in the desert or a rainforest). We recommend using subclasses of EnvO’s biome class:  http://purl.obolibrary.org/obo/ENVO_00000428. EnvO documentation about how to use the field: https://github.com/EnvironmentOntology/envo/wiki/Using-ENVO-with-MIxS</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2050,7 +2086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR1"/>
+  <dimension ref="A1:AP1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2061,203 +2097,209 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Local Environmental Context</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Environmental Medium</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Broad-Scale Environmental Context</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Sample storage location</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Sample storage setting</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Sample storage address</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Elevation (meters)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Environmental Medium</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Site Type</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Sample type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Water depth (m)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Site Type</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Local Environmental Context</t>
-        </is>
-      </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Sample Supertype</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Country/Ocean</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Longitude</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Latitude</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Country/Ocean</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Sampling depth (discrete, cm)</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>QR Code</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>City/Town/Lake/Location</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Region/Province/State</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Age Estimate (to, KABP)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Sampling depth estimation (bottom, cm)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Link to other relevant data</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Link to images</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Miscellaneous Environmental Measurements or Observations</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Miscellaneous Sample Measurements or Observations</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Disposal date</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Sampling Site</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Running Project Title</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Sampling Date</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Age Estimate (from, KABP)</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Period Estimate</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Sampling Method</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Sample provider(s)</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Sediment type</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>PI (KU ID)</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Correlation depth (top, cm)</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Correlation depth (bottom, cm)</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Grant</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Sampling depth estimation (top, cm)</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Storing date</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Grant</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>PI (KU ID)</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Age Estimate (from, KABP)</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Period Estimate</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Marine isotope stage estimate</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Sediment type</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Sampling Date</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Correlation depth (top, cm)</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Correlation depth (bottom, cm)</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>Sample provider(s)</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>Sampling depth estimation (top, cm)</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>Sampling depth (discrete, cm)</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>Running Project Title</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>City/Town/Lake/Location</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>Sampling Site</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr"/>
-      <c r="AP1" s="1" t="inlineStr"/>
-      <c r="AQ1" s="1" t="inlineStr"/>
-      <c r="AR1" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>